<commit_message>
Correcciones para templates y lectura de db con valores vacios o nulos
</commit_message>
<xml_diff>
--- a/data/database/templates.xlsx
+++ b/data/database/templates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,47 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>updated_at</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>config_path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ETL Simce Estudiantes Lenguaje</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Plantilla importada desde simce_estudiantes_lenguaje.json</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ETL Archivo</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>{"variables_documento":{},"secciones_fijas":[],"secciones_dinamicas":[],"etlParams":[{"id":"header_row","type":"text","label":"Fila Encabezado","value":"23","config":{"id":"header_row","label":"Fila Encabezado","type":"text","limit":1}},{"id":"output_name","type":"text","label":"Nombre Salida","value":"simce_2025_estudiantes.xlsx","config":{"id":"output_name","label":"Nombre Salida","type":"text","limit":1}},{"id":"select_columns","type":"list_text","label":"Seleccionar Columnas","value":["Nombre","RUT","Curso","B","M","O","Puntaje","Rend","SIMCE","Nota","Logro"],"config":{"id":"select_columns","label":"Seleccionar Columnas","type":"list_text","limit":0}},{"id":"rename_columns","type":"list_pair","label":"Renombrar Columnas","value":[{"key":"B","val":"Buenas"},{"key":"M","val":"Malas"},{"key":"O","val":"Omitidas"},{"key":"Rend","val":"Rendimiento"},{"key":"SIMCE","val":"SIMCE"},{"key":"Nota","val":"Nota"},{"key":"Logro","val":"Nivel de Logro"}],"config":{"id":"rename_columns","label":"Renombrar Columnas","type":"list_pair","limit":0,"fields":["Original","Final"]}},{"id":"enrich_data","type":"list_pair","label":"Enriquecer Data","value":[{"key":"Año","val":"2025"},{"key":"Asignatura","val":"Lenguaje"},{"key":"Mes","val":"Noviembre"},{"key":"Número_Prueba","val":"5"}],"config":{"id":"enrich_data","label":"Enriquecer Data","type":"list_pair","limit":0,"fields":["Columna","Valor"]}}]}</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-02-10 00:30:10</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>template001.json</t>
         </is>
       </c>
     </row>

</xml_diff>